<commit_message>
Update Course Planner template
</commit_message>
<xml_diff>
--- a/DV Course Planner Template.xlsx
+++ b/DV Course Planner Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hariharan_chipedge\Music\engg-automation-git-file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15785E0A-6F0D-4C2E-A3D0-37BD873854A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C5BE0AE-B681-41DA-BAF8-B7E09937C55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="162">
   <si>
     <t>Assessments / Soft Skills Session : Fridays</t>
   </si>
@@ -406,12 +406,6 @@
     <t>UVM phases and categorization</t>
   </si>
   <si>
-    <t>Holiday (Ganesha Chaturthi)</t>
-  </si>
-  <si>
-    <t>Holiday</t>
-  </si>
-  <si>
     <t>Digital Design</t>
   </si>
   <si>
@@ -452,9 +446,6 @@
     <t>Sequence, Sequencer Driver hand shake mechanism</t>
   </si>
   <si>
-    <t>Holiday(Gandhi Jayanthi)</t>
-  </si>
-  <si>
     <t>Blocking &amp; Non-Blocking methods</t>
   </si>
   <si>
@@ -482,9 +473,6 @@
   </si>
   <si>
     <t>Module Level Assessment - UVM</t>
-  </si>
-  <si>
-    <t>Holiday (Dussera)</t>
   </si>
   <si>
     <t>AXI4-Lite Theory (Project)</t>
@@ -650,7 +638,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -685,18 +673,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC9DAF8"/>
         <bgColor rgb="FFC9DAF8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA4C2F4"/>
-        <bgColor rgb="FFA4C2F4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9FC5E8"/>
-        <bgColor rgb="FF9FC5E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -1044,7 +1020,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1113,200 +1089,196 @@
     <xf numFmtId="164" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1527,7 +1499,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W160"/>
+  <dimension ref="A1:W158"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
@@ -1543,67 +1515,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="107" t="s">
-        <v>163</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="54"/>
+      <c r="A1" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="108" t="s">
-        <v>164</v>
-      </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="40"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="111" t="s">
-        <v>165</v>
-      </c>
-      <c r="G2" s="38" t="s">
+      <c r="A2" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" s="41"/>
+      <c r="C2" s="45"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="H2" s="38"/>
-      <c r="I2" s="37" t="s">
-        <v>162</v>
+      <c r="G2" s="104" t="s">
+        <v>157</v>
+      </c>
+      <c r="H2" s="104"/>
+      <c r="I2" s="103" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="32.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="108" t="s">
+      <c r="A3" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="112"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="37"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="103"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="72" t="s">
+      <c r="B4" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="74" t="s">
+      <c r="C4" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="43"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="109"/>
-      <c r="G4" s="67" t="s">
+      <c r="D4" s="41"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="91" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="68"/>
-      <c r="I4" s="56"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="84"/>
     </row>
     <row r="5" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="48"/>
@@ -1611,10 +1583,10 @@
       <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="110" t="s">
+      <c r="D5" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="40"/>
+      <c r="E5" s="45"/>
       <c r="F5" s="47"/>
       <c r="G5" s="1" t="s">
         <v>5</v>
@@ -1627,15 +1599,15 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A6" s="52">
+      <c r="A6" s="51">
         <v>1</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="63" t="s">
+      <c r="D6" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="40"/>
+      <c r="E6" s="45"/>
       <c r="F6" s="47"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1647,10 +1619,10 @@
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="D7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="40"/>
+      <c r="E7" s="45"/>
       <c r="F7" s="47"/>
       <c r="G7" s="6" t="s">
         <v>10</v>
@@ -1668,10 +1640,10 @@
       <c r="C8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="63" t="s">
+      <c r="D8" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="40"/>
+      <c r="E8" s="45"/>
       <c r="F8" s="47"/>
       <c r="G8" s="6" t="s">
         <v>10</v>
@@ -1689,10 +1661,10 @@
       <c r="C9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="40"/>
+      <c r="E9" s="45"/>
       <c r="F9" s="47"/>
       <c r="G9" s="6" t="s">
         <v>10</v>
@@ -1710,10 +1682,10 @@
       <c r="C10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="63" t="s">
+      <c r="D10" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="40"/>
+      <c r="E10" s="45"/>
       <c r="F10" s="47"/>
       <c r="G10" s="6" t="s">
         <v>10</v>
@@ -1726,30 +1698,30 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="40"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="45"/>
       <c r="F11" s="47"/>
-      <c r="G11" s="70"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="40"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="45"/>
     </row>
     <row r="12" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="52">
+      <c r="A12" s="51">
         <v>2</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="63" t="s">
+      <c r="D12" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="40"/>
+      <c r="E12" s="45"/>
       <c r="F12" s="47"/>
       <c r="G12" s="6" t="s">
         <v>18</v>
@@ -1767,10 +1739,10 @@
       <c r="C13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="40"/>
+      <c r="E13" s="45"/>
       <c r="F13" s="47"/>
       <c r="G13" s="6" t="s">
         <v>18</v>
@@ -1788,10 +1760,10 @@
       <c r="C14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="40"/>
+      <c r="E14" s="45"/>
       <c r="F14" s="47"/>
       <c r="G14" s="6" t="s">
         <v>18</v>
@@ -1809,10 +1781,10 @@
       <c r="C15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="71" t="s">
+      <c r="D15" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="40"/>
+      <c r="E15" s="45"/>
       <c r="F15" s="47"/>
       <c r="G15" s="6" t="s">
         <v>18</v>
@@ -1830,10 +1802,10 @@
       <c r="C16" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="71" t="s">
+      <c r="D16" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="40"/>
+      <c r="E16" s="45"/>
       <c r="F16" s="47"/>
       <c r="G16" s="6" t="s">
         <v>18</v>
@@ -1846,30 +1818,30 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="73" t="s">
+      <c r="A17" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="40"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="45"/>
       <c r="F17" s="47"/>
-      <c r="G17" s="70"/>
-      <c r="H17" s="43"/>
-      <c r="I17" s="40"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="45"/>
     </row>
     <row r="18" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A18" s="52">
+      <c r="A18" s="51">
         <v>3</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="40"/>
+      <c r="E18" s="45"/>
       <c r="F18" s="47"/>
       <c r="G18" s="6" t="s">
         <v>22</v>
@@ -1887,10 +1859,10 @@
       <c r="C19" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="40"/>
+      <c r="E19" s="45"/>
       <c r="F19" s="47"/>
       <c r="G19" s="6" t="s">
         <v>22</v>
@@ -1908,10 +1880,10 @@
       <c r="C20" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D20" s="63" t="s">
+      <c r="D20" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="40"/>
+      <c r="E20" s="45"/>
       <c r="F20" s="47"/>
       <c r="G20" s="6" t="s">
         <v>22</v>
@@ -1929,10 +1901,10 @@
       <c r="C21" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="40"/>
+      <c r="E21" s="45"/>
       <c r="F21" s="47"/>
       <c r="G21" s="6" t="s">
         <v>22</v>
@@ -1950,10 +1922,10 @@
       <c r="C22" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="D22" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="40"/>
+      <c r="E22" s="45"/>
       <c r="F22" s="47"/>
       <c r="G22" s="6" t="s">
         <v>22</v>
@@ -1966,30 +1938,30 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="40"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="45"/>
       <c r="F23" s="47"/>
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
       <c r="I23" s="14"/>
     </row>
     <row r="24" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="52">
+      <c r="A24" s="51">
         <v>1</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="40"/>
+      <c r="E24" s="45"/>
       <c r="F24" s="47"/>
       <c r="G24" s="6" t="s">
         <v>10</v>
@@ -2007,10 +1979,10 @@
       <c r="C25" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="64" t="s">
+      <c r="D25" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="E25" s="40"/>
+      <c r="E25" s="45"/>
       <c r="F25" s="47"/>
       <c r="G25" s="6" t="s">
         <v>10</v>
@@ -2028,10 +2000,10 @@
       <c r="C26" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="64" t="s">
+      <c r="D26" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="40"/>
+      <c r="E26" s="45"/>
       <c r="F26" s="47"/>
       <c r="G26" s="6" t="s">
         <v>10</v>
@@ -2049,10 +2021,10 @@
       <c r="C27" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="64" t="s">
+      <c r="D27" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="E27" s="40"/>
+      <c r="E27" s="45"/>
       <c r="F27" s="47"/>
       <c r="G27" s="6" t="s">
         <v>10</v>
@@ -2070,10 +2042,10 @@
       <c r="C28" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="64" t="s">
+      <c r="D28" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="E28" s="40"/>
+      <c r="E28" s="45"/>
       <c r="F28" s="48"/>
       <c r="G28" s="6" t="s">
         <v>10</v>
@@ -2086,36 +2058,36 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="43"/>
-      <c r="C29" s="43"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="43"/>
-      <c r="I29" s="40"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="41"/>
+      <c r="I29" s="45"/>
     </row>
     <row r="30" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A30" s="52">
+      <c r="A30" s="51">
         <v>2</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D30" s="65" t="s">
+      <c r="D30" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="E30" s="40"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="66" t="s">
+      <c r="E30" s="45"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="H30" s="43"/>
-      <c r="I30" s="40"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="45"/>
     </row>
     <row r="31" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A31" s="47"/>
@@ -2123,16 +2095,16 @@
       <c r="C31" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="65" t="s">
+      <c r="D31" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="E31" s="40"/>
+      <c r="E31" s="45"/>
       <c r="F31" s="47"/>
-      <c r="G31" s="66" t="s">
+      <c r="G31" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="H31" s="43"/>
-      <c r="I31" s="40"/>
+      <c r="H31" s="41"/>
+      <c r="I31" s="45"/>
     </row>
     <row r="32" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A32" s="47"/>
@@ -2140,16 +2112,16 @@
       <c r="C32" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="E32" s="40"/>
+      <c r="E32" s="45"/>
       <c r="F32" s="47"/>
-      <c r="G32" s="66" t="s">
+      <c r="G32" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="H32" s="43"/>
-      <c r="I32" s="40"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="45"/>
     </row>
     <row r="33" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A33" s="47"/>
@@ -2157,16 +2129,16 @@
       <c r="C33" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="40"/>
+      <c r="E33" s="45"/>
       <c r="F33" s="47"/>
-      <c r="G33" s="66" t="s">
+      <c r="G33" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="43"/>
-      <c r="I33" s="40"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="45"/>
     </row>
     <row r="34" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A34" s="48"/>
@@ -2174,48 +2146,48 @@
       <c r="C34" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="E34" s="40"/>
+      <c r="E34" s="45"/>
       <c r="F34" s="48"/>
-      <c r="G34" s="60" t="s">
+      <c r="G34" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="43"/>
-      <c r="I34" s="40"/>
+      <c r="H34" s="41"/>
+      <c r="I34" s="45"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="45" t="s">
+      <c r="A35" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="43"/>
-      <c r="C35" s="43"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="40"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
+      <c r="I35" s="45"/>
     </row>
     <row r="36" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A36" s="52">
+      <c r="A36" s="51">
         <v>3</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="41" t="s">
+      <c r="D36" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="E36" s="40"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="66" t="s">
+      <c r="E36" s="45"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="H36" s="43"/>
-      <c r="I36" s="40"/>
+      <c r="H36" s="41"/>
+      <c r="I36" s="45"/>
     </row>
     <row r="37" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A37" s="47"/>
@@ -2223,16 +2195,16 @@
       <c r="C37" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D37" s="41" t="s">
+      <c r="D37" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="40"/>
+      <c r="E37" s="45"/>
       <c r="F37" s="47"/>
-      <c r="G37" s="66" t="s">
+      <c r="G37" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="H37" s="43"/>
-      <c r="I37" s="40"/>
+      <c r="H37" s="41"/>
+      <c r="I37" s="45"/>
     </row>
     <row r="38" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A38" s="47"/>
@@ -2240,16 +2212,16 @@
       <c r="C38" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D38" s="103" t="s">
+      <c r="D38" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="40"/>
+      <c r="E38" s="45"/>
       <c r="F38" s="47"/>
-      <c r="G38" s="66" t="s">
+      <c r="G38" s="55" t="s">
         <v>50</v>
       </c>
-      <c r="H38" s="43"/>
-      <c r="I38" s="40"/>
+      <c r="H38" s="41"/>
+      <c r="I38" s="45"/>
     </row>
     <row r="39" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A39" s="47"/>
@@ -2257,16 +2229,16 @@
       <c r="C39" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D39" s="41" t="s">
+      <c r="D39" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="40"/>
+      <c r="E39" s="45"/>
       <c r="F39" s="47"/>
-      <c r="G39" s="66" t="s">
+      <c r="G39" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="H39" s="43"/>
-      <c r="I39" s="40"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="45"/>
     </row>
     <row r="40" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A40" s="48"/>
@@ -2274,48 +2246,48 @@
       <c r="C40" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D40" s="104" t="s">
+      <c r="D40" s="54" t="s">
         <v>53</v>
       </c>
-      <c r="E40" s="40"/>
+      <c r="E40" s="45"/>
       <c r="F40" s="48"/>
-      <c r="G40" s="60" t="s">
+      <c r="G40" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="H40" s="43"/>
-      <c r="I40" s="40"/>
+      <c r="H40" s="41"/>
+      <c r="I40" s="45"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="45" t="s">
+      <c r="A41" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B41" s="43"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="40"/>
+      <c r="B41" s="41"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="41"/>
+      <c r="I41" s="45"/>
     </row>
     <row r="42" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A42" s="52">
+      <c r="A42" s="51">
         <v>4</v>
       </c>
       <c r="B42" s="12"/>
       <c r="C42" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D42" s="41" t="s">
+      <c r="D42" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="E42" s="40"/>
-      <c r="F42" s="52"/>
-      <c r="G42" s="41" t="s">
+      <c r="E42" s="45"/>
+      <c r="F42" s="51"/>
+      <c r="G42" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="H42" s="43"/>
-      <c r="I42" s="40"/>
+      <c r="H42" s="41"/>
+      <c r="I42" s="45"/>
     </row>
     <row r="43" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A43" s="47"/>
@@ -2323,16 +2295,16 @@
       <c r="C43" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D43" s="41" t="s">
+      <c r="D43" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="E43" s="40"/>
+      <c r="E43" s="45"/>
       <c r="F43" s="47"/>
-      <c r="G43" s="41" t="s">
+      <c r="G43" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="H43" s="43"/>
-      <c r="I43" s="40"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="45"/>
     </row>
     <row r="44" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A44" s="47"/>
@@ -2340,16 +2312,16 @@
       <c r="C44" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D44" s="41" t="s">
+      <c r="D44" s="52" t="s">
         <v>59</v>
       </c>
-      <c r="E44" s="40"/>
+      <c r="E44" s="45"/>
       <c r="F44" s="47"/>
-      <c r="G44" s="66" t="s">
+      <c r="G44" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="H44" s="43"/>
-      <c r="I44" s="40"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="45"/>
     </row>
     <row r="45" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A45" s="47"/>
@@ -2357,16 +2329,16 @@
       <c r="C45" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D45" s="41" t="s">
+      <c r="D45" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="E45" s="40"/>
+      <c r="E45" s="45"/>
       <c r="F45" s="47"/>
-      <c r="G45" s="66" t="s">
+      <c r="G45" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="H45" s="43"/>
-      <c r="I45" s="40"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="45"/>
     </row>
     <row r="46" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A46" s="48"/>
@@ -2374,48 +2346,48 @@
       <c r="C46" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D46" s="41" t="s">
+      <c r="D46" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E46" s="40"/>
+      <c r="E46" s="45"/>
       <c r="F46" s="48"/>
-      <c r="G46" s="60" t="s">
+      <c r="G46" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="43"/>
-      <c r="I46" s="40"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="45"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="45" t="s">
+      <c r="A47" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B47" s="43"/>
-      <c r="C47" s="43"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="43"/>
-      <c r="H47" s="43"/>
-      <c r="I47" s="40"/>
+      <c r="B47" s="41"/>
+      <c r="C47" s="41"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="41"/>
+      <c r="F47" s="41"/>
+      <c r="G47" s="41"/>
+      <c r="H47" s="41"/>
+      <c r="I47" s="45"/>
     </row>
     <row r="48" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A48" s="52">
+      <c r="A48" s="51">
         <v>5</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D48" s="41" t="s">
+      <c r="D48" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="E48" s="40"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="66" t="s">
+      <c r="E48" s="45"/>
+      <c r="F48" s="51"/>
+      <c r="G48" s="55" t="s">
         <v>65</v>
       </c>
-      <c r="H48" s="43"/>
-      <c r="I48" s="40"/>
+      <c r="H48" s="41"/>
+      <c r="I48" s="45"/>
     </row>
     <row r="49" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A49" s="47"/>
@@ -2423,16 +2395,16 @@
       <c r="C49" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D49" s="41" t="s">
+      <c r="D49" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="E49" s="40"/>
+      <c r="E49" s="45"/>
       <c r="F49" s="47"/>
-      <c r="G49" s="66" t="s">
+      <c r="G49" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="H49" s="43"/>
-      <c r="I49" s="40"/>
+      <c r="H49" s="41"/>
+      <c r="I49" s="45"/>
     </row>
     <row r="50" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A50" s="47"/>
@@ -2440,16 +2412,16 @@
       <c r="C50" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D50" s="41" t="s">
+      <c r="D50" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="E50" s="40"/>
+      <c r="E50" s="45"/>
       <c r="F50" s="47"/>
-      <c r="G50" s="66" t="s">
+      <c r="G50" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="H50" s="43"/>
-      <c r="I50" s="40"/>
+      <c r="H50" s="41"/>
+      <c r="I50" s="45"/>
     </row>
     <row r="51" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A51" s="47"/>
@@ -2457,16 +2429,16 @@
       <c r="C51" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D51" s="41" t="s">
+      <c r="D51" s="52" t="s">
         <v>69</v>
       </c>
-      <c r="E51" s="40"/>
+      <c r="E51" s="45"/>
       <c r="F51" s="47"/>
-      <c r="G51" s="66" t="s">
+      <c r="G51" s="55" t="s">
         <v>70</v>
       </c>
-      <c r="H51" s="43"/>
-      <c r="I51" s="40"/>
+      <c r="H51" s="41"/>
+      <c r="I51" s="45"/>
     </row>
     <row r="52" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A52" s="48"/>
@@ -2474,48 +2446,48 @@
       <c r="C52" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D52" s="41" t="s">
+      <c r="D52" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="E52" s="40"/>
+      <c r="E52" s="45"/>
       <c r="F52" s="48"/>
-      <c r="G52" s="60" t="s">
+      <c r="G52" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H52" s="43"/>
-      <c r="I52" s="40"/>
+      <c r="H52" s="41"/>
+      <c r="I52" s="45"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="45" t="s">
+      <c r="A53" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B53" s="43"/>
-      <c r="C53" s="43"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="43"/>
-      <c r="I53" s="40"/>
+      <c r="B53" s="41"/>
+      <c r="C53" s="41"/>
+      <c r="D53" s="41"/>
+      <c r="E53" s="41"/>
+      <c r="F53" s="41"/>
+      <c r="G53" s="41"/>
+      <c r="H53" s="41"/>
+      <c r="I53" s="45"/>
     </row>
     <row r="54" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A54" s="52">
+      <c r="A54" s="51">
         <v>6</v>
       </c>
       <c r="B54" s="12"/>
       <c r="C54" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D54" s="60" t="s">
+      <c r="D54" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="E54" s="61"/>
+      <c r="E54" s="66"/>
       <c r="F54" s="19"/>
-      <c r="G54" s="104" t="s">
-        <v>74</v>
-      </c>
-      <c r="H54" s="43"/>
-      <c r="I54" s="61"/>
+      <c r="G54" s="54" t="s">
+        <v>74</v>
+      </c>
+      <c r="H54" s="41"/>
+      <c r="I54" s="66"/>
     </row>
     <row r="55" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A55" s="47"/>
@@ -2523,16 +2495,16 @@
       <c r="C55" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D55" s="41" t="s">
+      <c r="D55" s="52" t="s">
         <v>75</v>
       </c>
-      <c r="E55" s="40"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H55" s="43"/>
-      <c r="I55" s="40"/>
+      <c r="E55" s="45"/>
+      <c r="F55" s="51"/>
+      <c r="G55" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H55" s="41"/>
+      <c r="I55" s="45"/>
     </row>
     <row r="56" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A56" s="47"/>
@@ -2540,16 +2512,16 @@
       <c r="C56" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D56" s="41" t="s">
+      <c r="D56" s="52" t="s">
         <v>76</v>
       </c>
-      <c r="E56" s="40"/>
+      <c r="E56" s="45"/>
       <c r="F56" s="47"/>
-      <c r="G56" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H56" s="43"/>
-      <c r="I56" s="40"/>
+      <c r="G56" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H56" s="41"/>
+      <c r="I56" s="45"/>
     </row>
     <row r="57" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A57" s="47"/>
@@ -2557,16 +2529,16 @@
       <c r="C57" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D57" s="41" t="s">
+      <c r="D57" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="E57" s="40"/>
+      <c r="E57" s="45"/>
       <c r="F57" s="48"/>
-      <c r="G57" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H57" s="43"/>
-      <c r="I57" s="40"/>
+      <c r="G57" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H57" s="41"/>
+      <c r="I57" s="45"/>
     </row>
     <row r="58" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A58" s="48"/>
@@ -2574,48 +2546,48 @@
       <c r="C58" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D58" s="39" t="s">
+      <c r="D58" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="E58" s="61"/>
+      <c r="E58" s="66"/>
       <c r="F58" s="20"/>
-      <c r="G58" s="105" t="s">
+      <c r="G58" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="H58" s="43"/>
-      <c r="I58" s="40"/>
+      <c r="H58" s="41"/>
+      <c r="I58" s="45"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="45" t="s">
+      <c r="A59" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="43"/>
-      <c r="C59" s="43"/>
-      <c r="D59" s="43"/>
-      <c r="E59" s="43"/>
-      <c r="F59" s="43"/>
-      <c r="G59" s="43"/>
-      <c r="H59" s="43"/>
-      <c r="I59" s="40"/>
+      <c r="B59" s="41"/>
+      <c r="C59" s="41"/>
+      <c r="D59" s="41"/>
+      <c r="E59" s="41"/>
+      <c r="F59" s="41"/>
+      <c r="G59" s="41"/>
+      <c r="H59" s="41"/>
+      <c r="I59" s="45"/>
     </row>
     <row r="60" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A60" s="52">
+      <c r="A60" s="51">
         <v>7</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D60" s="41" t="s">
+      <c r="D60" s="52" t="s">
         <v>79</v>
       </c>
-      <c r="E60" s="40"/>
-      <c r="F60" s="106"/>
-      <c r="G60" s="39" t="s">
-        <v>74</v>
-      </c>
-      <c r="H60" s="43"/>
-      <c r="I60" s="40"/>
+      <c r="E60" s="45"/>
+      <c r="F60" s="64"/>
+      <c r="G60" s="67" t="s">
+        <v>74</v>
+      </c>
+      <c r="H60" s="41"/>
+      <c r="I60" s="45"/>
     </row>
     <row r="61" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A61" s="47"/>
@@ -2623,16 +2595,16 @@
       <c r="C61" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D61" s="41" t="s">
+      <c r="D61" s="52" t="s">
         <v>80</v>
       </c>
-      <c r="E61" s="40"/>
+      <c r="E61" s="45"/>
       <c r="F61" s="47"/>
-      <c r="G61" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H61" s="43"/>
-      <c r="I61" s="40"/>
+      <c r="G61" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H61" s="41"/>
+      <c r="I61" s="45"/>
     </row>
     <row r="62" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A62" s="47"/>
@@ -2640,16 +2612,16 @@
       <c r="C62" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D62" s="41" t="s">
+      <c r="D62" s="52" t="s">
         <v>81</v>
       </c>
-      <c r="E62" s="40"/>
+      <c r="E62" s="45"/>
       <c r="F62" s="47"/>
-      <c r="G62" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H62" s="43"/>
-      <c r="I62" s="40"/>
+      <c r="G62" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H62" s="41"/>
+      <c r="I62" s="45"/>
     </row>
     <row r="63" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A63" s="47"/>
@@ -2657,16 +2629,16 @@
       <c r="C63" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D63" s="41" t="s">
+      <c r="D63" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="E63" s="40"/>
+      <c r="E63" s="45"/>
       <c r="F63" s="47"/>
-      <c r="G63" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="H63" s="43"/>
-      <c r="I63" s="40"/>
+      <c r="G63" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="H63" s="41"/>
+      <c r="I63" s="45"/>
     </row>
     <row r="64" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A64" s="48"/>
@@ -2674,48 +2646,48 @@
       <c r="C64" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D64" s="103" t="s">
+      <c r="D64" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="E64" s="40"/>
+      <c r="E64" s="45"/>
       <c r="F64" s="48"/>
-      <c r="G64" s="60" t="s">
+      <c r="G64" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H64" s="43"/>
-      <c r="I64" s="40"/>
+      <c r="H64" s="41"/>
+      <c r="I64" s="45"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="45" t="s">
+      <c r="A65" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B65" s="43"/>
-      <c r="C65" s="43"/>
-      <c r="D65" s="43"/>
-      <c r="E65" s="43"/>
-      <c r="F65" s="43"/>
-      <c r="G65" s="43"/>
-      <c r="H65" s="43"/>
-      <c r="I65" s="40"/>
+      <c r="B65" s="41"/>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+      <c r="E65" s="41"/>
+      <c r="F65" s="41"/>
+      <c r="G65" s="41"/>
+      <c r="H65" s="41"/>
+      <c r="I65" s="45"/>
     </row>
     <row r="66" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A66" s="52">
+      <c r="A66" s="51">
         <v>8</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D66" s="59" t="s">
+      <c r="D66" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="E66" s="40"/>
-      <c r="F66" s="50"/>
-      <c r="G66" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H66" s="43"/>
-      <c r="I66" s="40"/>
+      <c r="E66" s="45"/>
+      <c r="F66" s="65"/>
+      <c r="G66" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H66" s="41"/>
+      <c r="I66" s="45"/>
     </row>
     <row r="67" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A67" s="47"/>
@@ -2723,16 +2695,16 @@
       <c r="C67" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D67" s="59" t="s">
+      <c r="D67" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="E67" s="40"/>
+      <c r="E67" s="45"/>
       <c r="F67" s="47"/>
-      <c r="G67" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H67" s="43"/>
-      <c r="I67" s="40"/>
+      <c r="G67" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H67" s="41"/>
+      <c r="I67" s="45"/>
     </row>
     <row r="68" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A68" s="47"/>
@@ -2740,16 +2712,16 @@
       <c r="C68" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D68" s="59" t="s">
+      <c r="D68" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="E68" s="40"/>
+      <c r="E68" s="45"/>
       <c r="F68" s="47"/>
-      <c r="G68" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H68" s="43"/>
-      <c r="I68" s="40"/>
+      <c r="G68" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H68" s="41"/>
+      <c r="I68" s="45"/>
     </row>
     <row r="69" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A69" s="47"/>
@@ -2757,16 +2729,16 @@
       <c r="C69" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D69" s="59" t="s">
+      <c r="D69" s="61" t="s">
         <v>87</v>
       </c>
-      <c r="E69" s="40"/>
+      <c r="E69" s="45"/>
       <c r="F69" s="47"/>
-      <c r="G69" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H69" s="43"/>
-      <c r="I69" s="40"/>
+      <c r="G69" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H69" s="41"/>
+      <c r="I69" s="45"/>
     </row>
     <row r="70" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A70" s="48"/>
@@ -2774,48 +2746,48 @@
       <c r="C70" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D70" s="41" t="s">
+      <c r="D70" s="52" t="s">
         <v>88</v>
       </c>
-      <c r="E70" s="40"/>
+      <c r="E70" s="45"/>
       <c r="F70" s="48"/>
-      <c r="G70" s="60" t="s">
+      <c r="G70" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H70" s="43"/>
-      <c r="I70" s="40"/>
+      <c r="H70" s="41"/>
+      <c r="I70" s="45"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="45" t="s">
+      <c r="A71" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B71" s="43"/>
-      <c r="C71" s="43"/>
-      <c r="D71" s="43"/>
-      <c r="E71" s="43"/>
-      <c r="F71" s="43"/>
-      <c r="G71" s="43"/>
-      <c r="H71" s="43"/>
-      <c r="I71" s="40"/>
+      <c r="B71" s="41"/>
+      <c r="C71" s="41"/>
+      <c r="D71" s="41"/>
+      <c r="E71" s="41"/>
+      <c r="F71" s="41"/>
+      <c r="G71" s="41"/>
+      <c r="H71" s="41"/>
+      <c r="I71" s="45"/>
     </row>
     <row r="72" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A72" s="52">
+      <c r="A72" s="51">
         <v>9</v>
       </c>
       <c r="B72" s="12"/>
       <c r="C72" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D72" s="59" t="s">
+      <c r="D72" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="E72" s="40"/>
-      <c r="F72" s="50"/>
-      <c r="G72" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H72" s="43"/>
-      <c r="I72" s="40"/>
+      <c r="E72" s="45"/>
+      <c r="F72" s="65"/>
+      <c r="G72" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H72" s="41"/>
+      <c r="I72" s="45"/>
     </row>
     <row r="73" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A73" s="47"/>
@@ -2823,16 +2795,16 @@
       <c r="C73" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D73" s="59" t="s">
+      <c r="D73" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="E73" s="40"/>
+      <c r="E73" s="45"/>
       <c r="F73" s="47"/>
-      <c r="G73" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H73" s="43"/>
-      <c r="I73" s="40"/>
+      <c r="G73" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H73" s="41"/>
+      <c r="I73" s="45"/>
     </row>
     <row r="74" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A74" s="47"/>
@@ -2840,16 +2812,16 @@
       <c r="C74" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D74" s="59" t="s">
+      <c r="D74" s="61" t="s">
         <v>91</v>
       </c>
-      <c r="E74" s="40"/>
+      <c r="E74" s="45"/>
       <c r="F74" s="47"/>
-      <c r="G74" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H74" s="43"/>
-      <c r="I74" s="40"/>
+      <c r="G74" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H74" s="41"/>
+      <c r="I74" s="45"/>
     </row>
     <row r="75" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A75" s="47"/>
@@ -2857,16 +2829,16 @@
       <c r="C75" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D75" s="59" t="s">
+      <c r="D75" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="E75" s="40"/>
+      <c r="E75" s="45"/>
       <c r="F75" s="47"/>
-      <c r="G75" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H75" s="43"/>
-      <c r="I75" s="40"/>
+      <c r="G75" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H75" s="41"/>
+      <c r="I75" s="45"/>
     </row>
     <row r="76" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A76" s="48"/>
@@ -2874,48 +2846,48 @@
       <c r="C76" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D76" s="39" t="s">
+      <c r="D76" s="67" t="s">
         <v>93</v>
       </c>
-      <c r="E76" s="40"/>
+      <c r="E76" s="45"/>
       <c r="F76" s="48"/>
-      <c r="G76" s="60" t="s">
+      <c r="G76" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="H76" s="43"/>
-      <c r="I76" s="40"/>
+      <c r="H76" s="41"/>
+      <c r="I76" s="45"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="45" t="s">
+      <c r="A77" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B77" s="43"/>
-      <c r="C77" s="43"/>
-      <c r="D77" s="43"/>
-      <c r="E77" s="43"/>
-      <c r="F77" s="43"/>
-      <c r="G77" s="43"/>
-      <c r="H77" s="43"/>
-      <c r="I77" s="40"/>
+      <c r="B77" s="41"/>
+      <c r="C77" s="41"/>
+      <c r="D77" s="41"/>
+      <c r="E77" s="41"/>
+      <c r="F77" s="41"/>
+      <c r="G77" s="41"/>
+      <c r="H77" s="41"/>
+      <c r="I77" s="45"/>
     </row>
     <row r="78" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A78" s="52">
+      <c r="A78" s="51">
         <v>10</v>
       </c>
       <c r="B78" s="12"/>
       <c r="C78" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D78" s="59" t="s">
+      <c r="D78" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="E78" s="40"/>
-      <c r="F78" s="50"/>
-      <c r="G78" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H78" s="43"/>
-      <c r="I78" s="40"/>
+      <c r="E78" s="45"/>
+      <c r="F78" s="65"/>
+      <c r="G78" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H78" s="41"/>
+      <c r="I78" s="45"/>
     </row>
     <row r="79" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A79" s="47"/>
@@ -2923,16 +2895,16 @@
       <c r="C79" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D79" s="59" t="s">
+      <c r="D79" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="E79" s="40"/>
+      <c r="E79" s="45"/>
       <c r="F79" s="47"/>
-      <c r="G79" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H79" s="43"/>
-      <c r="I79" s="40"/>
+      <c r="G79" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H79" s="41"/>
+      <c r="I79" s="45"/>
     </row>
     <row r="80" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A80" s="47"/>
@@ -2940,16 +2912,16 @@
       <c r="C80" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D80" s="59" t="s">
+      <c r="D80" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="E80" s="40"/>
+      <c r="E80" s="45"/>
       <c r="F80" s="47"/>
-      <c r="G80" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H80" s="43"/>
-      <c r="I80" s="40"/>
+      <c r="G80" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H80" s="41"/>
+      <c r="I80" s="45"/>
     </row>
     <row r="81" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A81" s="47"/>
@@ -2957,16 +2929,16 @@
       <c r="C81" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D81" s="59" t="s">
+      <c r="D81" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="E81" s="40"/>
+      <c r="E81" s="45"/>
       <c r="F81" s="47"/>
-      <c r="G81" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H81" s="43"/>
-      <c r="I81" s="40"/>
+      <c r="G81" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H81" s="41"/>
+      <c r="I81" s="45"/>
     </row>
     <row r="82" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A82" s="48"/>
@@ -2974,48 +2946,48 @@
       <c r="C82" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D82" s="59" t="s">
+      <c r="D82" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="E82" s="40"/>
+      <c r="E82" s="45"/>
       <c r="F82" s="48"/>
-      <c r="G82" s="60" t="s">
+      <c r="G82" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H82" s="43"/>
-      <c r="I82" s="40"/>
+      <c r="H82" s="41"/>
+      <c r="I82" s="45"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A83" s="45" t="s">
+      <c r="A83" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B83" s="43"/>
-      <c r="C83" s="43"/>
-      <c r="D83" s="43"/>
-      <c r="E83" s="43"/>
-      <c r="F83" s="43"/>
-      <c r="G83" s="43"/>
-      <c r="H83" s="43"/>
-      <c r="I83" s="40"/>
+      <c r="B83" s="41"/>
+      <c r="C83" s="41"/>
+      <c r="D83" s="41"/>
+      <c r="E83" s="41"/>
+      <c r="F83" s="41"/>
+      <c r="G83" s="41"/>
+      <c r="H83" s="41"/>
+      <c r="I83" s="45"/>
     </row>
     <row r="84" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A84" s="52">
+      <c r="A84" s="51">
         <v>11</v>
       </c>
       <c r="B84" s="12"/>
       <c r="C84" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D84" s="59" t="s">
+      <c r="D84" s="61" t="s">
         <v>100</v>
       </c>
-      <c r="E84" s="40"/>
-      <c r="F84" s="50"/>
-      <c r="G84" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H84" s="43"/>
-      <c r="I84" s="40"/>
+      <c r="E84" s="45"/>
+      <c r="F84" s="65"/>
+      <c r="G84" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H84" s="41"/>
+      <c r="I84" s="45"/>
       <c r="J84" s="21" t="s">
         <v>101</v>
       </c>
@@ -3026,16 +2998,16 @@
       <c r="C85" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D85" s="59" t="s">
+      <c r="D85" s="61" t="s">
         <v>102</v>
       </c>
-      <c r="E85" s="40"/>
+      <c r="E85" s="45"/>
       <c r="F85" s="47"/>
-      <c r="G85" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H85" s="43"/>
-      <c r="I85" s="40"/>
+      <c r="G85" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H85" s="41"/>
+      <c r="I85" s="45"/>
     </row>
     <row r="86" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A86" s="47"/>
@@ -3043,16 +3015,16 @@
       <c r="C86" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D86" s="59" t="s">
+      <c r="D86" s="61" t="s">
         <v>103</v>
       </c>
-      <c r="E86" s="40"/>
+      <c r="E86" s="45"/>
       <c r="F86" s="47"/>
-      <c r="G86" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H86" s="43"/>
-      <c r="I86" s="40"/>
+      <c r="G86" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H86" s="41"/>
+      <c r="I86" s="45"/>
     </row>
     <row r="87" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A87" s="47"/>
@@ -3060,16 +3032,16 @@
       <c r="C87" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D87" s="59" t="s">
+      <c r="D87" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="E87" s="40"/>
+      <c r="E87" s="45"/>
       <c r="F87" s="47"/>
-      <c r="G87" s="59" t="s">
+      <c r="G87" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="H87" s="43"/>
-      <c r="I87" s="40"/>
+      <c r="H87" s="41"/>
+      <c r="I87" s="45"/>
     </row>
     <row r="88" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A88" s="48"/>
@@ -3077,46 +3049,46 @@
       <c r="C88" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D88" s="60" t="s">
+      <c r="D88" s="56" t="s">
         <v>106</v>
       </c>
-      <c r="E88" s="40"/>
+      <c r="E88" s="45"/>
       <c r="F88" s="48"/>
-      <c r="G88" s="60" t="s">
+      <c r="G88" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H88" s="43"/>
-      <c r="I88" s="40"/>
+      <c r="H88" s="41"/>
+      <c r="I88" s="45"/>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A89" s="45" t="s">
+      <c r="A89" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B89" s="43"/>
-      <c r="C89" s="43"/>
-      <c r="D89" s="43"/>
-      <c r="E89" s="43"/>
-      <c r="F89" s="43"/>
-      <c r="G89" s="43"/>
-      <c r="H89" s="43"/>
-      <c r="I89" s="40"/>
+      <c r="B89" s="41"/>
+      <c r="C89" s="41"/>
+      <c r="D89" s="41"/>
+      <c r="E89" s="41"/>
+      <c r="F89" s="41"/>
+      <c r="G89" s="41"/>
+      <c r="H89" s="41"/>
+      <c r="I89" s="45"/>
     </row>
     <row r="90" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A90" s="52">
+      <c r="A90" s="51">
         <v>12</v>
       </c>
       <c r="B90" s="12"/>
       <c r="C90" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D90" s="60" t="s">
+      <c r="D90" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="E90" s="43"/>
-      <c r="F90" s="43"/>
-      <c r="G90" s="43"/>
-      <c r="H90" s="43"/>
-      <c r="I90" s="40"/>
+      <c r="E90" s="41"/>
+      <c r="F90" s="41"/>
+      <c r="G90" s="41"/>
+      <c r="H90" s="41"/>
+      <c r="I90" s="45"/>
     </row>
     <row r="91" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A91" s="47"/>
@@ -3124,16 +3096,16 @@
       <c r="C91" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D91" s="59" t="s">
+      <c r="D91" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="E91" s="40"/>
-      <c r="F91" s="50"/>
-      <c r="G91" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H91" s="43"/>
-      <c r="I91" s="40"/>
+      <c r="E91" s="45"/>
+      <c r="F91" s="65"/>
+      <c r="G91" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H91" s="41"/>
+      <c r="I91" s="45"/>
     </row>
     <row r="92" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A92" s="47"/>
@@ -3141,16 +3113,16 @@
       <c r="C92" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D92" s="39" t="s">
+      <c r="D92" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="E92" s="40"/>
+      <c r="E92" s="45"/>
       <c r="F92" s="47"/>
-      <c r="G92" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H92" s="43"/>
-      <c r="I92" s="40"/>
+      <c r="G92" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H92" s="41"/>
+      <c r="I92" s="45"/>
     </row>
     <row r="93" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A93" s="47"/>
@@ -3158,16 +3130,16 @@
       <c r="C93" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D93" s="59" t="s">
+      <c r="D93" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="E93" s="40"/>
+      <c r="E93" s="45"/>
       <c r="F93" s="47"/>
-      <c r="G93" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H93" s="43"/>
-      <c r="I93" s="40"/>
+      <c r="G93" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H93" s="41"/>
+      <c r="I93" s="45"/>
     </row>
     <row r="94" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A94" s="48"/>
@@ -3175,48 +3147,48 @@
       <c r="C94" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D94" s="59" t="s">
+      <c r="D94" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="E94" s="40"/>
+      <c r="E94" s="45"/>
       <c r="F94" s="48"/>
-      <c r="G94" s="60" t="s">
+      <c r="G94" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H94" s="43"/>
-      <c r="I94" s="40"/>
+      <c r="H94" s="41"/>
+      <c r="I94" s="45"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A95" s="45" t="s">
+      <c r="A95" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B95" s="43"/>
-      <c r="C95" s="43"/>
-      <c r="D95" s="43"/>
-      <c r="E95" s="43"/>
-      <c r="F95" s="43"/>
-      <c r="G95" s="43"/>
-      <c r="H95" s="43"/>
-      <c r="I95" s="40"/>
+      <c r="B95" s="41"/>
+      <c r="C95" s="41"/>
+      <c r="D95" s="41"/>
+      <c r="E95" s="41"/>
+      <c r="F95" s="41"/>
+      <c r="G95" s="41"/>
+      <c r="H95" s="41"/>
+      <c r="I95" s="45"/>
     </row>
     <row r="96" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A96" s="52">
+      <c r="A96" s="51">
         <v>13</v>
       </c>
       <c r="B96" s="12"/>
       <c r="C96" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D96" s="59" t="s">
+      <c r="D96" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="E96" s="40"/>
-      <c r="F96" s="50"/>
-      <c r="G96" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H96" s="43"/>
-      <c r="I96" s="40"/>
+      <c r="E96" s="45"/>
+      <c r="F96" s="65"/>
+      <c r="G96" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H96" s="41"/>
+      <c r="I96" s="45"/>
     </row>
     <row r="97" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A97" s="47"/>
@@ -3224,16 +3196,16 @@
       <c r="C97" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D97" s="59" t="s">
+      <c r="D97" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="E97" s="40"/>
+      <c r="E97" s="45"/>
       <c r="F97" s="47"/>
-      <c r="G97" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H97" s="43"/>
-      <c r="I97" s="40"/>
+      <c r="G97" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H97" s="41"/>
+      <c r="I97" s="45"/>
     </row>
     <row r="98" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A98" s="47"/>
@@ -3241,16 +3213,16 @@
       <c r="C98" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D98" s="59" t="s">
+      <c r="D98" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="E98" s="40"/>
+      <c r="E98" s="45"/>
       <c r="F98" s="47"/>
-      <c r="G98" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H98" s="43"/>
-      <c r="I98" s="40"/>
+      <c r="G98" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H98" s="41"/>
+      <c r="I98" s="45"/>
     </row>
     <row r="99" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A99" s="47"/>
@@ -3258,16 +3230,16 @@
       <c r="C99" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D99" s="59" t="s">
+      <c r="D99" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="E99" s="40"/>
+      <c r="E99" s="45"/>
       <c r="F99" s="47"/>
-      <c r="G99" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H99" s="43"/>
-      <c r="I99" s="40"/>
+      <c r="G99" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H99" s="41"/>
+      <c r="I99" s="45"/>
     </row>
     <row r="100" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A100" s="48"/>
@@ -3275,57 +3247,57 @@
       <c r="C100" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D100" s="59" t="s">
+      <c r="D100" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="E100" s="40"/>
+      <c r="E100" s="45"/>
       <c r="F100" s="48"/>
-      <c r="G100" s="59" t="s">
+      <c r="G100" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="H100" s="43"/>
-      <c r="I100" s="40"/>
+      <c r="H100" s="41"/>
+      <c r="I100" s="45"/>
     </row>
     <row r="101" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A101" s="45" t="s">
+      <c r="A101" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B101" s="43"/>
-      <c r="C101" s="43"/>
-      <c r="D101" s="43"/>
-      <c r="E101" s="43"/>
-      <c r="F101" s="43"/>
-      <c r="G101" s="43"/>
-      <c r="H101" s="43"/>
-      <c r="I101" s="40"/>
+      <c r="B101" s="41"/>
+      <c r="C101" s="41"/>
+      <c r="D101" s="41"/>
+      <c r="E101" s="41"/>
+      <c r="F101" s="41"/>
+      <c r="G101" s="41"/>
+      <c r="H101" s="41"/>
+      <c r="I101" s="45"/>
     </row>
     <row r="102" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A102" s="52">
+      <c r="A102" s="51">
         <v>14</v>
       </c>
       <c r="B102" s="12"/>
       <c r="C102" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D102" s="59" t="s">
+      <c r="D102" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="E102" s="40"/>
-      <c r="F102" s="50"/>
-      <c r="G102" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H102" s="43"/>
-      <c r="I102" s="40"/>
-      <c r="J102" s="98"/>
+      <c r="E102" s="45"/>
+      <c r="F102" s="65"/>
+      <c r="G102" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H102" s="41"/>
+      <c r="I102" s="45"/>
+      <c r="J102" s="71"/>
       <c r="K102" s="22"/>
       <c r="L102" s="23"/>
-      <c r="M102" s="94"/>
-      <c r="N102" s="87"/>
-      <c r="O102" s="95"/>
-      <c r="P102" s="94"/>
-      <c r="Q102" s="86"/>
-      <c r="R102" s="87"/>
+      <c r="M102" s="70"/>
+      <c r="N102" s="69"/>
+      <c r="O102" s="74"/>
+      <c r="P102" s="70"/>
+      <c r="Q102" s="73"/>
+      <c r="R102" s="69"/>
     </row>
     <row r="103" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A103" s="47"/>
@@ -3333,25 +3305,25 @@
       <c r="C103" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D103" s="59" t="s">
+      <c r="D103" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="E103" s="40"/>
+      <c r="E103" s="45"/>
       <c r="F103" s="47"/>
-      <c r="G103" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H103" s="43"/>
-      <c r="I103" s="40"/>
-      <c r="J103" s="99"/>
+      <c r="G103" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H103" s="41"/>
+      <c r="I103" s="45"/>
+      <c r="J103" s="72"/>
       <c r="K103" s="22"/>
       <c r="L103" s="23"/>
-      <c r="M103" s="94"/>
-      <c r="N103" s="87"/>
-      <c r="O103" s="96"/>
-      <c r="P103" s="94"/>
-      <c r="Q103" s="86"/>
-      <c r="R103" s="87"/>
+      <c r="M103" s="70"/>
+      <c r="N103" s="69"/>
+      <c r="O103" s="75"/>
+      <c r="P103" s="70"/>
+      <c r="Q103" s="73"/>
+      <c r="R103" s="69"/>
     </row>
     <row r="104" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A104" s="47"/>
@@ -3359,25 +3331,25 @@
       <c r="C104" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D104" s="100" t="s">
+      <c r="D104" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="E104" s="40"/>
+      <c r="E104" s="45"/>
       <c r="F104" s="47"/>
-      <c r="G104" s="100" t="s">
-        <v>74</v>
-      </c>
-      <c r="H104" s="43"/>
-      <c r="I104" s="40"/>
-      <c r="J104" s="99"/>
+      <c r="G104" s="77" t="s">
+        <v>74</v>
+      </c>
+      <c r="H104" s="41"/>
+      <c r="I104" s="45"/>
+      <c r="J104" s="72"/>
       <c r="K104" s="26"/>
       <c r="L104" s="27"/>
-      <c r="M104" s="101"/>
-      <c r="N104" s="87"/>
-      <c r="O104" s="96"/>
-      <c r="P104" s="101"/>
-      <c r="Q104" s="86"/>
-      <c r="R104" s="87"/>
+      <c r="M104" s="68"/>
+      <c r="N104" s="69"/>
+      <c r="O104" s="75"/>
+      <c r="P104" s="68"/>
+      <c r="Q104" s="73"/>
+      <c r="R104" s="69"/>
       <c r="S104" s="28"/>
       <c r="T104" s="28"/>
       <c r="U104" s="28"/>
@@ -3390,25 +3362,25 @@
       <c r="C105" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D105" s="59" t="s">
+      <c r="D105" s="61" t="s">
         <v>123</v>
       </c>
-      <c r="E105" s="40"/>
+      <c r="E105" s="45"/>
       <c r="F105" s="47"/>
-      <c r="G105" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H105" s="43"/>
-      <c r="I105" s="40"/>
-      <c r="J105" s="99"/>
+      <c r="G105" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H105" s="41"/>
+      <c r="I105" s="45"/>
+      <c r="J105" s="72"/>
       <c r="K105" s="22"/>
       <c r="L105" s="23"/>
-      <c r="M105" s="94"/>
-      <c r="N105" s="87"/>
-      <c r="O105" s="96"/>
-      <c r="P105" s="94"/>
-      <c r="Q105" s="86"/>
-      <c r="R105" s="87"/>
+      <c r="M105" s="70"/>
+      <c r="N105" s="69"/>
+      <c r="O105" s="75"/>
+      <c r="P105" s="70"/>
+      <c r="Q105" s="73"/>
+      <c r="R105" s="69"/>
     </row>
     <row r="106" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A106" s="48"/>
@@ -3416,55 +3388,49 @@
       <c r="C106" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D106" s="41" t="s">
-        <v>74</v>
-      </c>
-      <c r="E106" s="40"/>
+      <c r="D106" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="E106" s="45"/>
       <c r="F106" s="48"/>
-      <c r="G106" s="60" t="s">
+      <c r="G106" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="H106" s="43"/>
-      <c r="I106" s="40"/>
-      <c r="J106" s="99"/>
+      <c r="H106" s="41"/>
+      <c r="I106" s="45"/>
+      <c r="J106" s="72"/>
       <c r="K106" s="22"/>
       <c r="L106" s="23"/>
-      <c r="M106" s="98"/>
-      <c r="N106" s="99"/>
-      <c r="O106" s="97"/>
-      <c r="P106" s="102"/>
-      <c r="Q106" s="86"/>
-      <c r="R106" s="87"/>
+      <c r="M106" s="71"/>
+      <c r="N106" s="72"/>
+      <c r="O106" s="76"/>
+      <c r="P106" s="78"/>
+      <c r="Q106" s="73"/>
+      <c r="R106" s="69"/>
     </row>
     <row r="107" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A107" s="45" t="s">
+      <c r="A107" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B107" s="43"/>
-      <c r="C107" s="43"/>
-      <c r="D107" s="43"/>
-      <c r="E107" s="43"/>
-      <c r="F107" s="43"/>
-      <c r="G107" s="43"/>
-      <c r="H107" s="43"/>
-      <c r="I107" s="40"/>
+      <c r="B107" s="41"/>
+      <c r="C107" s="41"/>
+      <c r="D107" s="41"/>
+      <c r="E107" s="41"/>
+      <c r="F107" s="41"/>
+      <c r="G107" s="41"/>
+      <c r="H107" s="41"/>
+      <c r="I107" s="45"/>
     </row>
     <row r="108" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A108" s="62">
-        <v>15</v>
-      </c>
+      <c r="A108" s="106"/>
       <c r="B108" s="29"/>
-      <c r="C108" s="90" t="s">
-        <v>124</v>
-      </c>
-      <c r="D108" s="43"/>
-      <c r="E108" s="40"/>
-      <c r="F108" s="91"/>
-      <c r="G108" s="84" t="s">
-        <v>125</v>
-      </c>
-      <c r="H108" s="43"/>
-      <c r="I108" s="40"/>
+      <c r="C108" s="110"/>
+      <c r="D108" s="37"/>
+      <c r="E108" s="36"/>
+      <c r="F108" s="107"/>
+      <c r="G108" s="111"/>
+      <c r="H108" s="108"/>
+      <c r="I108" s="109"/>
       <c r="J108" s="21"/>
       <c r="K108" s="21"/>
       <c r="L108" s="21"/>
@@ -3484,18 +3450,18 @@
       <c r="A109" s="47"/>
       <c r="B109" s="30"/>
       <c r="C109" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D109" s="79" t="s">
+        <v>125</v>
+      </c>
+      <c r="E109" s="80"/>
+      <c r="F109" s="47"/>
+      <c r="G109" s="61" t="s">
         <v>126</v>
       </c>
-      <c r="D109" s="92" t="s">
-        <v>127</v>
-      </c>
-      <c r="E109" s="93"/>
-      <c r="F109" s="47"/>
-      <c r="G109" s="59" t="s">
-        <v>128</v>
-      </c>
-      <c r="H109" s="43"/>
-      <c r="I109" s="40"/>
+      <c r="H109" s="41"/>
+      <c r="I109" s="45"/>
       <c r="J109" s="21"/>
       <c r="K109" s="21"/>
       <c r="L109" s="21"/>
@@ -3515,16 +3481,16 @@
       <c r="A110" s="47"/>
       <c r="B110" s="30"/>
       <c r="C110" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D110" s="79"/>
-      <c r="E110" s="80"/>
+        <v>124</v>
+      </c>
+      <c r="D110" s="81"/>
+      <c r="E110" s="82"/>
       <c r="F110" s="47"/>
-      <c r="G110" s="59" t="s">
+      <c r="G110" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="H110" s="43"/>
-      <c r="I110" s="40"/>
+      <c r="H110" s="41"/>
+      <c r="I110" s="45"/>
       <c r="J110" s="21"/>
       <c r="K110" s="21"/>
       <c r="L110" s="21"/>
@@ -3544,16 +3510,16 @@
       <c r="A111" s="47"/>
       <c r="B111" s="30"/>
       <c r="C111" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D111" s="79"/>
-      <c r="E111" s="80"/>
+        <v>124</v>
+      </c>
+      <c r="D111" s="81"/>
+      <c r="E111" s="82"/>
       <c r="F111" s="47"/>
-      <c r="G111" s="59" t="s">
+      <c r="G111" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="H111" s="43"/>
-      <c r="I111" s="40"/>
+      <c r="H111" s="41"/>
+      <c r="I111" s="45"/>
       <c r="J111" s="21"/>
       <c r="K111" s="21"/>
       <c r="L111" s="21"/>
@@ -3573,16 +3539,16 @@
       <c r="A112" s="48"/>
       <c r="B112" s="31"/>
       <c r="C112" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D112" s="55"/>
-      <c r="E112" s="56"/>
+        <v>124</v>
+      </c>
+      <c r="D112" s="83"/>
+      <c r="E112" s="84"/>
       <c r="F112" s="48"/>
-      <c r="G112" s="59" t="s">
+      <c r="G112" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="H112" s="43"/>
-      <c r="I112" s="40"/>
+      <c r="H112" s="41"/>
+      <c r="I112" s="45"/>
       <c r="J112" s="28"/>
       <c r="K112" s="28"/>
       <c r="L112" s="28"/>
@@ -3599,36 +3565,36 @@
       <c r="W112" s="28"/>
     </row>
     <row r="113" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A113" s="45" t="s">
+      <c r="A113" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B113" s="43"/>
-      <c r="C113" s="43"/>
-      <c r="D113" s="43"/>
-      <c r="E113" s="43"/>
-      <c r="F113" s="43"/>
-      <c r="G113" s="43"/>
-      <c r="H113" s="43"/>
-      <c r="I113" s="40"/>
+      <c r="B113" s="41"/>
+      <c r="C113" s="41"/>
+      <c r="D113" s="41"/>
+      <c r="E113" s="41"/>
+      <c r="F113" s="41"/>
+      <c r="G113" s="41"/>
+      <c r="H113" s="41"/>
+      <c r="I113" s="45"/>
     </row>
     <row r="114" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A114" s="52">
+      <c r="A114" s="51">
         <v>16</v>
       </c>
       <c r="B114" s="12"/>
       <c r="C114" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D114" s="59" t="s">
-        <v>129</v>
-      </c>
-      <c r="E114" s="40"/>
-      <c r="F114" s="50"/>
-      <c r="G114" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H114" s="43"/>
-      <c r="I114" s="40"/>
+      <c r="D114" s="61" t="s">
+        <v>127</v>
+      </c>
+      <c r="E114" s="45"/>
+      <c r="F114" s="65"/>
+      <c r="G114" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H114" s="41"/>
+      <c r="I114" s="45"/>
     </row>
     <row r="115" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A115" s="47"/>
@@ -3636,16 +3602,16 @@
       <c r="C115" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D115" s="59" t="s">
-        <v>130</v>
-      </c>
-      <c r="E115" s="40"/>
+      <c r="D115" s="61" t="s">
+        <v>128</v>
+      </c>
+      <c r="E115" s="45"/>
       <c r="F115" s="47"/>
-      <c r="G115" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H115" s="43"/>
-      <c r="I115" s="40"/>
+      <c r="G115" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H115" s="41"/>
+      <c r="I115" s="45"/>
     </row>
     <row r="116" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A116" s="47"/>
@@ -3653,16 +3619,16 @@
       <c r="C116" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D116" s="59" t="s">
-        <v>131</v>
-      </c>
-      <c r="E116" s="40"/>
+      <c r="D116" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="E116" s="45"/>
       <c r="F116" s="47"/>
-      <c r="G116" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H116" s="43"/>
-      <c r="I116" s="40"/>
+      <c r="G116" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H116" s="41"/>
+      <c r="I116" s="45"/>
     </row>
     <row r="117" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A117" s="47"/>
@@ -3670,16 +3636,16 @@
       <c r="C117" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D117" s="59" t="s">
-        <v>132</v>
-      </c>
-      <c r="E117" s="40"/>
+      <c r="D117" s="61" t="s">
+        <v>130</v>
+      </c>
+      <c r="E117" s="45"/>
       <c r="F117" s="47"/>
-      <c r="G117" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H117" s="43"/>
-      <c r="I117" s="40"/>
+      <c r="G117" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H117" s="41"/>
+      <c r="I117" s="45"/>
     </row>
     <row r="118" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A118" s="48"/>
@@ -3687,50 +3653,50 @@
       <c r="C118" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D118" s="41" t="s">
-        <v>74</v>
-      </c>
-      <c r="E118" s="40"/>
+      <c r="D118" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="E118" s="45"/>
       <c r="F118" s="48"/>
-      <c r="G118" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="H118" s="43"/>
-      <c r="I118" s="40"/>
+      <c r="G118" s="56" t="s">
+        <v>131</v>
+      </c>
+      <c r="H118" s="41"/>
+      <c r="I118" s="45"/>
     </row>
     <row r="119" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A119" s="45" t="s">
+      <c r="A119" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B119" s="43"/>
-      <c r="C119" s="43"/>
-      <c r="D119" s="43"/>
-      <c r="E119" s="43"/>
-      <c r="F119" s="43"/>
-      <c r="G119" s="43"/>
-      <c r="H119" s="43"/>
-      <c r="I119" s="40"/>
+      <c r="B119" s="41"/>
+      <c r="C119" s="41"/>
+      <c r="D119" s="41"/>
+      <c r="E119" s="41"/>
+      <c r="F119" s="41"/>
+      <c r="G119" s="41"/>
+      <c r="H119" s="41"/>
+      <c r="I119" s="45"/>
     </row>
     <row r="120" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A120" s="52">
+      <c r="A120" s="51">
         <v>17</v>
       </c>
       <c r="B120" s="12"/>
       <c r="C120" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D120" s="59" t="s">
-        <v>134</v>
-      </c>
-      <c r="E120" s="40"/>
-      <c r="F120" s="50"/>
-      <c r="G120" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H120" s="43"/>
-      <c r="I120" s="40"/>
+      <c r="D120" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="E120" s="45"/>
+      <c r="F120" s="65"/>
+      <c r="G120" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H120" s="41"/>
+      <c r="I120" s="45"/>
       <c r="J120" s="21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="121" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
@@ -3739,16 +3705,16 @@
       <c r="C121" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D121" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="E121" s="40"/>
+      <c r="D121" s="61" t="s">
+        <v>134</v>
+      </c>
+      <c r="E121" s="45"/>
       <c r="F121" s="47"/>
-      <c r="G121" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H121" s="43"/>
-      <c r="I121" s="40"/>
+      <c r="G121" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H121" s="41"/>
+      <c r="I121" s="45"/>
     </row>
     <row r="122" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A122" s="47"/>
@@ -3756,16 +3722,16 @@
       <c r="C122" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D122" s="39" t="s">
-        <v>137</v>
-      </c>
-      <c r="E122" s="40"/>
+      <c r="D122" s="67" t="s">
+        <v>135</v>
+      </c>
+      <c r="E122" s="45"/>
       <c r="F122" s="47"/>
-      <c r="G122" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H122" s="43"/>
-      <c r="I122" s="40"/>
+      <c r="G122" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H122" s="41"/>
+      <c r="I122" s="45"/>
     </row>
     <row r="123" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A123" s="47"/>
@@ -3773,79 +3739,75 @@
       <c r="C123" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D123" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="E123" s="40"/>
+      <c r="D123" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="E123" s="45"/>
       <c r="F123" s="47"/>
-      <c r="G123" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H123" s="43"/>
-      <c r="I123" s="40"/>
+      <c r="G123" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H123" s="41"/>
+      <c r="I123" s="45"/>
     </row>
     <row r="124" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A124" s="48"/>
-      <c r="B124" s="32"/>
-      <c r="C124" s="85" t="s">
-        <v>139</v>
-      </c>
-      <c r="D124" s="86"/>
-      <c r="E124" s="87"/>
-      <c r="F124" s="48"/>
-      <c r="G124" s="88" t="s">
-        <v>125</v>
-      </c>
-      <c r="H124" s="43"/>
-      <c r="I124" s="40"/>
+      <c r="A124" s="47"/>
+      <c r="B124" s="12"/>
+      <c r="C124" s="112"/>
+      <c r="D124" s="113"/>
+      <c r="E124" s="37"/>
+      <c r="F124" s="47"/>
+      <c r="G124" s="114"/>
+      <c r="H124" s="108"/>
+      <c r="I124" s="109"/>
     </row>
     <row r="125" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A125" s="45" t="s">
+      <c r="A125" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B125" s="43"/>
-      <c r="C125" s="43"/>
-      <c r="D125" s="43"/>
-      <c r="E125" s="43"/>
-      <c r="F125" s="43"/>
-      <c r="G125" s="43"/>
-      <c r="H125" s="43"/>
-      <c r="I125" s="40"/>
+      <c r="B125" s="41"/>
+      <c r="C125" s="41"/>
+      <c r="D125" s="41"/>
+      <c r="E125" s="41"/>
+      <c r="F125" s="41"/>
+      <c r="G125" s="41"/>
+      <c r="H125" s="41"/>
+      <c r="I125" s="45"/>
     </row>
     <row r="126" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A126" s="58">
+      <c r="A126" s="96">
         <v>18</v>
       </c>
       <c r="B126" s="16"/>
       <c r="C126" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D126" s="41" t="s">
-        <v>140</v>
-      </c>
-      <c r="E126" s="40"/>
-      <c r="F126" s="75" t="s">
-        <v>141</v>
-      </c>
-      <c r="G126" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="H126" s="43"/>
-      <c r="I126" s="40"/>
-      <c r="J126" s="33"/>
-      <c r="K126" s="33"/>
-      <c r="L126" s="33"/>
-      <c r="M126" s="33"/>
-      <c r="N126" s="33"/>
-      <c r="O126" s="33"/>
-      <c r="P126" s="33"/>
-      <c r="Q126" s="33"/>
-      <c r="R126" s="33"/>
-      <c r="S126" s="33"/>
-      <c r="T126" s="33"/>
-      <c r="U126" s="33"/>
-      <c r="V126" s="33"/>
-      <c r="W126" s="33"/>
+      <c r="D126" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="E126" s="45"/>
+      <c r="F126" s="97" t="s">
+        <v>138</v>
+      </c>
+      <c r="G126" s="86" t="s">
+        <v>74</v>
+      </c>
+      <c r="H126" s="41"/>
+      <c r="I126" s="45"/>
+      <c r="J126" s="32"/>
+      <c r="K126" s="32"/>
+      <c r="L126" s="32"/>
+      <c r="M126" s="32"/>
+      <c r="N126" s="32"/>
+      <c r="O126" s="32"/>
+      <c r="P126" s="32"/>
+      <c r="Q126" s="32"/>
+      <c r="R126" s="32"/>
+      <c r="S126" s="32"/>
+      <c r="T126" s="32"/>
+      <c r="U126" s="32"/>
+      <c r="V126" s="32"/>
+      <c r="W126" s="32"/>
     </row>
     <row r="127" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A127" s="47"/>
@@ -3853,16 +3815,16 @@
       <c r="C127" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D127" s="76" t="s">
-        <v>142</v>
-      </c>
-      <c r="E127" s="40"/>
+      <c r="D127" s="87" t="s">
+        <v>139</v>
+      </c>
+      <c r="E127" s="45"/>
       <c r="F127" s="47"/>
-      <c r="G127" s="76" t="s">
-        <v>74</v>
-      </c>
-      <c r="H127" s="43"/>
-      <c r="I127" s="40"/>
+      <c r="G127" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="H127" s="41"/>
+      <c r="I127" s="45"/>
     </row>
     <row r="128" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A128" s="47"/>
@@ -3870,16 +3832,16 @@
       <c r="C128" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D128" s="76" t="s">
-        <v>143</v>
-      </c>
-      <c r="E128" s="40"/>
+      <c r="D128" s="87" t="s">
+        <v>140</v>
+      </c>
+      <c r="E128" s="45"/>
       <c r="F128" s="47"/>
-      <c r="G128" s="76" t="s">
-        <v>74</v>
-      </c>
-      <c r="H128" s="43"/>
-      <c r="I128" s="40"/>
+      <c r="G128" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="H128" s="41"/>
+      <c r="I128" s="45"/>
     </row>
     <row r="129" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A129" s="47"/>
@@ -3887,16 +3849,16 @@
       <c r="C129" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D129" s="76" t="s">
-        <v>144</v>
-      </c>
-      <c r="E129" s="40"/>
+      <c r="D129" s="87" t="s">
+        <v>141</v>
+      </c>
+      <c r="E129" s="45"/>
       <c r="F129" s="47"/>
-      <c r="G129" s="76" t="s">
-        <v>74</v>
-      </c>
-      <c r="H129" s="43"/>
-      <c r="I129" s="40"/>
+      <c r="G129" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="H129" s="41"/>
+      <c r="I129" s="45"/>
     </row>
     <row r="130" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A130" s="48"/>
@@ -3904,140 +3866,138 @@
       <c r="C130" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D130" s="77" t="s">
-        <v>74</v>
-      </c>
-      <c r="E130" s="40"/>
+      <c r="D130" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="E130" s="45"/>
       <c r="F130" s="48"/>
-      <c r="G130" s="81" t="s">
-        <v>145</v>
-      </c>
-      <c r="H130" s="43"/>
-      <c r="I130" s="40"/>
+      <c r="G130" s="90" t="s">
+        <v>142</v>
+      </c>
+      <c r="H130" s="41"/>
+      <c r="I130" s="45"/>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" s="45" t="s">
+      <c r="A131" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B131" s="43"/>
-      <c r="C131" s="43"/>
-      <c r="D131" s="43"/>
-      <c r="E131" s="43"/>
-      <c r="F131" s="43"/>
-      <c r="G131" s="43"/>
-      <c r="H131" s="43"/>
-      <c r="I131" s="40"/>
+      <c r="B131" s="41"/>
+      <c r="C131" s="41"/>
+      <c r="D131" s="41"/>
+      <c r="E131" s="41"/>
+      <c r="F131" s="41"/>
+      <c r="G131" s="41"/>
+      <c r="H131" s="41"/>
+      <c r="I131" s="45"/>
     </row>
     <row r="132" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A132" s="52">
+      <c r="A132" s="51">
         <v>19</v>
       </c>
       <c r="B132" s="12"/>
       <c r="C132" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D132" s="78" t="s">
-        <v>146</v>
-      </c>
-      <c r="E132" s="54"/>
-      <c r="F132" s="50"/>
-      <c r="G132" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="H132" s="43"/>
-      <c r="I132" s="40"/>
+        <v>124</v>
+      </c>
+      <c r="D132" s="89" t="s">
+        <v>143</v>
+      </c>
+      <c r="E132" s="43"/>
+      <c r="F132" s="65"/>
+      <c r="G132" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="H132" s="41"/>
+      <c r="I132" s="45"/>
     </row>
     <row r="133" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A133" s="47"/>
       <c r="B133" s="12"/>
       <c r="C133" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D133" s="79"/>
-      <c r="E133" s="80"/>
+        <v>124</v>
+      </c>
+      <c r="D133" s="81"/>
+      <c r="E133" s="82"/>
       <c r="F133" s="47"/>
-      <c r="G133" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="H133" s="43"/>
-      <c r="I133" s="40"/>
+      <c r="G133" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="H133" s="41"/>
+      <c r="I133" s="45"/>
     </row>
     <row r="134" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A134" s="47"/>
       <c r="B134" s="12"/>
       <c r="C134" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D134" s="79"/>
-      <c r="E134" s="80"/>
+        <v>124</v>
+      </c>
+      <c r="D134" s="81"/>
+      <c r="E134" s="82"/>
       <c r="F134" s="47"/>
-      <c r="G134" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="H134" s="43"/>
-      <c r="I134" s="40"/>
+      <c r="G134" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="H134" s="41"/>
+      <c r="I134" s="45"/>
     </row>
     <row r="135" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A135" s="47"/>
       <c r="B135" s="12"/>
       <c r="C135" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D135" s="55"/>
-      <c r="E135" s="56"/>
+        <v>124</v>
+      </c>
+      <c r="D135" s="83"/>
+      <c r="E135" s="84"/>
       <c r="F135" s="48"/>
-      <c r="G135" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="H135" s="43"/>
-      <c r="I135" s="40"/>
+      <c r="G135" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="H135" s="41"/>
+      <c r="I135" s="45"/>
     </row>
     <row r="136" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A136" s="48"/>
       <c r="B136" s="12"/>
       <c r="C136" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D136" s="60" t="s">
-        <v>148</v>
-      </c>
-      <c r="E136" s="43"/>
-      <c r="F136" s="43"/>
-      <c r="G136" s="43"/>
-      <c r="H136" s="43"/>
-      <c r="I136" s="40"/>
+        <v>124</v>
+      </c>
+      <c r="D136" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="E136" s="41"/>
+      <c r="F136" s="41"/>
+      <c r="G136" s="41"/>
+      <c r="H136" s="41"/>
+      <c r="I136" s="45"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A137" s="45" t="s">
+      <c r="A137" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B137" s="43"/>
-      <c r="C137" s="43"/>
-      <c r="D137" s="43"/>
-      <c r="E137" s="43"/>
-      <c r="F137" s="43"/>
-      <c r="G137" s="43"/>
-      <c r="H137" s="43"/>
-      <c r="I137" s="40"/>
+      <c r="B137" s="41"/>
+      <c r="C137" s="41"/>
+      <c r="D137" s="41"/>
+      <c r="E137" s="41"/>
+      <c r="F137" s="41"/>
+      <c r="G137" s="41"/>
+      <c r="H137" s="41"/>
+      <c r="I137" s="45"/>
     </row>
     <row r="138" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A138" s="52">
-        <v>20</v>
-      </c>
+      <c r="A138" s="47"/>
       <c r="B138" s="12"/>
       <c r="C138" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D138" s="53" t="s">
-        <v>149</v>
-      </c>
-      <c r="E138" s="54"/>
-      <c r="F138" s="50"/>
-      <c r="G138" s="82" t="s">
-        <v>149</v>
-      </c>
-      <c r="H138" s="83"/>
-      <c r="I138" s="54"/>
+      <c r="D138" s="99" t="s">
+        <v>146</v>
+      </c>
+      <c r="E138" s="45"/>
+      <c r="F138" s="47"/>
+      <c r="G138" s="100" t="s">
+        <v>144</v>
+      </c>
+      <c r="H138" s="41"/>
+      <c r="I138" s="45"/>
     </row>
     <row r="139" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A139" s="47"/>
@@ -4045,354 +4005,623 @@
       <c r="C139" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D139" s="55"/>
-      <c r="E139" s="56"/>
+      <c r="D139" s="99" t="s">
+        <v>71</v>
+      </c>
+      <c r="E139" s="45"/>
       <c r="F139" s="47"/>
-      <c r="G139" s="55"/>
-      <c r="H139" s="68"/>
-      <c r="I139" s="56"/>
+      <c r="G139" s="100" t="s">
+        <v>144</v>
+      </c>
+      <c r="H139" s="41"/>
+      <c r="I139" s="45"/>
     </row>
     <row r="140" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A140" s="47"/>
+      <c r="A140" s="48"/>
       <c r="B140" s="12"/>
       <c r="C140" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="D140" s="57" t="s">
-        <v>150</v>
-      </c>
-      <c r="E140" s="40"/>
-      <c r="F140" s="47"/>
-      <c r="G140" s="49" t="s">
         <v>147</v>
       </c>
-      <c r="H140" s="43"/>
-      <c r="I140" s="40"/>
-    </row>
-    <row r="141" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A141" s="47"/>
-      <c r="B141" s="12"/>
-      <c r="C141" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="D141" s="57" t="s">
-        <v>71</v>
-      </c>
-      <c r="E141" s="40"/>
-      <c r="F141" s="47"/>
-      <c r="G141" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="H141" s="43"/>
-      <c r="I141" s="40"/>
+      <c r="D140" s="98" t="s">
+        <v>148</v>
+      </c>
+      <c r="E140" s="45"/>
+      <c r="F140" s="48"/>
+      <c r="G140" s="100" t="s">
+        <v>149</v>
+      </c>
+      <c r="H140" s="41"/>
+      <c r="I140" s="45"/>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A141" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="B141" s="41"/>
+      <c r="C141" s="41"/>
+      <c r="D141" s="41"/>
+      <c r="E141" s="41"/>
+      <c r="F141" s="41"/>
+      <c r="G141" s="41"/>
+      <c r="H141" s="41"/>
+      <c r="I141" s="45"/>
     </row>
     <row r="142" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A142" s="48"/>
+      <c r="A142" s="51">
+        <v>21</v>
+      </c>
       <c r="B142" s="12"/>
       <c r="C142" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="D142" s="98" t="s">
+        <v>150</v>
+      </c>
+      <c r="E142" s="45"/>
+      <c r="F142" s="105"/>
+      <c r="G142" s="101" t="s">
+        <v>71</v>
+      </c>
+      <c r="H142" s="41"/>
+      <c r="I142" s="45"/>
+    </row>
+    <row r="143" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A143" s="47"/>
+      <c r="B143" s="12"/>
+      <c r="C143" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D143" s="98" t="s">
         <v>151</v>
       </c>
-      <c r="D142" s="51" t="s">
-        <v>152</v>
-      </c>
-      <c r="E142" s="40"/>
-      <c r="F142" s="48"/>
-      <c r="G142" s="49" t="s">
-        <v>153</v>
-      </c>
-      <c r="H142" s="43"/>
-      <c r="I142" s="40"/>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="B143" s="43"/>
-      <c r="C143" s="43"/>
-      <c r="D143" s="43"/>
-      <c r="E143" s="43"/>
-      <c r="F143" s="43"/>
-      <c r="G143" s="43"/>
-      <c r="H143" s="43"/>
-      <c r="I143" s="40"/>
+      <c r="E143" s="45"/>
+      <c r="F143" s="47"/>
+      <c r="G143" s="101" t="s">
+        <v>71</v>
+      </c>
+      <c r="H143" s="41"/>
+      <c r="I143" s="45"/>
     </row>
     <row r="144" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A144" s="52">
-        <v>21</v>
-      </c>
+      <c r="A144" s="47"/>
       <c r="B144" s="12"/>
       <c r="C144" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="D144" s="51" t="s">
-        <v>154</v>
-      </c>
-      <c r="E144" s="40"/>
-      <c r="F144" s="46"/>
-      <c r="G144" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="H144" s="43"/>
-      <c r="I144" s="40"/>
+        <v>147</v>
+      </c>
+      <c r="D144" s="98" t="s">
+        <v>152</v>
+      </c>
+      <c r="E144" s="45"/>
+      <c r="F144" s="47"/>
+      <c r="G144" s="101" t="s">
+        <v>153</v>
+      </c>
+      <c r="H144" s="41"/>
+      <c r="I144" s="45"/>
     </row>
     <row r="145" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A145" s="47"/>
       <c r="B145" s="12"/>
       <c r="C145" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="D145" s="51" t="s">
+        <v>154</v>
+      </c>
+      <c r="D145" s="67" t="s">
         <v>155</v>
       </c>
-      <c r="E145" s="40"/>
+      <c r="E145" s="45"/>
       <c r="F145" s="47"/>
-      <c r="G145" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="H145" s="43"/>
-      <c r="I145" s="40"/>
+      <c r="G145" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H145" s="41"/>
+      <c r="I145" s="45"/>
     </row>
     <row r="146" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A146" s="47"/>
+      <c r="A146" s="48"/>
       <c r="B146" s="12"/>
       <c r="C146" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="D146" s="51" t="s">
-        <v>156</v>
-      </c>
-      <c r="E146" s="40"/>
-      <c r="F146" s="47"/>
-      <c r="G146" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="H146" s="43"/>
-      <c r="I146" s="40"/>
-    </row>
-    <row r="147" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A147" s="47"/>
-      <c r="B147" s="12"/>
-      <c r="C147" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D147" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="E147" s="40"/>
-      <c r="F147" s="47"/>
-      <c r="G147" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H147" s="43"/>
-      <c r="I147" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D146" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E146" s="45"/>
+      <c r="F146" s="48"/>
+      <c r="G146" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H146" s="41"/>
+      <c r="I146" s="45"/>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A147" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="B147" s="41"/>
+      <c r="C147" s="41"/>
+      <c r="D147" s="41"/>
+      <c r="E147" s="41"/>
+      <c r="F147" s="41"/>
+      <c r="G147" s="41"/>
+      <c r="H147" s="41"/>
+      <c r="I147" s="45"/>
     </row>
     <row r="148" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A148" s="48"/>
+      <c r="A148" s="51">
+        <v>22</v>
+      </c>
       <c r="B148" s="12"/>
       <c r="C148" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D148" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E148" s="40"/>
-      <c r="F148" s="48"/>
-      <c r="G148" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H148" s="43"/>
-      <c r="I148" s="40"/>
-    </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A149" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="B149" s="43"/>
-      <c r="C149" s="43"/>
-      <c r="D149" s="43"/>
-      <c r="E149" s="43"/>
-      <c r="F149" s="43"/>
-      <c r="G149" s="43"/>
-      <c r="H149" s="43"/>
-      <c r="I149" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D148" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E148" s="45"/>
+      <c r="F148" s="105"/>
+      <c r="G148" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H148" s="41"/>
+      <c r="I148" s="45"/>
+    </row>
+    <row r="149" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A149" s="47"/>
+      <c r="B149" s="12"/>
+      <c r="C149" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D149" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E149" s="45"/>
+      <c r="F149" s="47"/>
+      <c r="G149" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H149" s="41"/>
+      <c r="I149" s="45"/>
     </row>
     <row r="150" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A150" s="52">
-        <v>22</v>
-      </c>
+      <c r="A150" s="47"/>
       <c r="B150" s="12"/>
       <c r="C150" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D150" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E150" s="40"/>
-      <c r="F150" s="46"/>
-      <c r="G150" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H150" s="43"/>
-      <c r="I150" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D150" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E150" s="45"/>
+      <c r="F150" s="47"/>
+      <c r="G150" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H150" s="41"/>
+      <c r="I150" s="45"/>
     </row>
     <row r="151" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A151" s="47"/>
       <c r="B151" s="12"/>
       <c r="C151" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D151" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E151" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D151" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E151" s="45"/>
       <c r="F151" s="47"/>
-      <c r="G151" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H151" s="43"/>
-      <c r="I151" s="40"/>
+      <c r="G151" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H151" s="41"/>
+      <c r="I151" s="45"/>
     </row>
     <row r="152" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A152" s="47"/>
+      <c r="A152" s="48"/>
       <c r="B152" s="12"/>
       <c r="C152" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D152" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E152" s="40"/>
-      <c r="F152" s="47"/>
-      <c r="G152" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H152" s="43"/>
-      <c r="I152" s="40"/>
-    </row>
-    <row r="153" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A153" s="47"/>
-      <c r="B153" s="12"/>
-      <c r="C153" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D153" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E153" s="40"/>
-      <c r="F153" s="47"/>
-      <c r="G153" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H153" s="43"/>
-      <c r="I153" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D152" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E152" s="45"/>
+      <c r="F152" s="48"/>
+      <c r="G152" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H152" s="41"/>
+      <c r="I152" s="45"/>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A153" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="B153" s="41"/>
+      <c r="C153" s="41"/>
+      <c r="D153" s="41"/>
+      <c r="E153" s="41"/>
+      <c r="F153" s="41"/>
+      <c r="G153" s="41"/>
+      <c r="H153" s="41"/>
+      <c r="I153" s="45"/>
     </row>
     <row r="154" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A154" s="48"/>
+      <c r="A154" s="51">
+        <v>23</v>
+      </c>
       <c r="B154" s="12"/>
       <c r="C154" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D154" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E154" s="40"/>
-      <c r="F154" s="48"/>
-      <c r="G154" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H154" s="43"/>
-      <c r="I154" s="40"/>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A155" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="B155" s="43"/>
-      <c r="C155" s="43"/>
-      <c r="D155" s="43"/>
-      <c r="E155" s="43"/>
-      <c r="F155" s="43"/>
-      <c r="G155" s="43"/>
-      <c r="H155" s="43"/>
-      <c r="I155" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D154" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E154" s="45"/>
+      <c r="F154" s="105"/>
+      <c r="G154" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H154" s="41"/>
+      <c r="I154" s="45"/>
+    </row>
+    <row r="155" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A155" s="47"/>
+      <c r="B155" s="12"/>
+      <c r="C155" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D155" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E155" s="45"/>
+      <c r="F155" s="47"/>
+      <c r="G155" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="H155" s="41"/>
+      <c r="I155" s="45"/>
     </row>
     <row r="156" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A156" s="52">
-        <v>23</v>
-      </c>
+      <c r="A156" s="47"/>
       <c r="B156" s="12"/>
       <c r="C156" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D156" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E156" s="40"/>
-      <c r="F156" s="46"/>
-      <c r="G156" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H156" s="43"/>
-      <c r="I156" s="40"/>
+        <v>154</v>
+      </c>
+      <c r="D156" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="E156" s="45"/>
+      <c r="F156" s="47"/>
+      <c r="G156" s="102" t="s">
+        <v>156</v>
+      </c>
+      <c r="H156" s="41"/>
+      <c r="I156" s="45"/>
     </row>
     <row r="157" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A157" s="47"/>
       <c r="B157" s="12"/>
-      <c r="C157" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D157" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E157" s="40"/>
+      <c r="C157" s="18"/>
+      <c r="D157" s="52"/>
+      <c r="E157" s="45"/>
       <c r="F157" s="47"/>
-      <c r="G157" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="H157" s="43"/>
-      <c r="I157" s="40"/>
+      <c r="G157" s="102"/>
+      <c r="H157" s="41"/>
+      <c r="I157" s="45"/>
     </row>
     <row r="158" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A158" s="47"/>
+      <c r="A158" s="48"/>
       <c r="B158" s="12"/>
-      <c r="C158" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="D158" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="E158" s="40"/>
-      <c r="F158" s="47"/>
-      <c r="G158" s="42" t="s">
-        <v>160</v>
-      </c>
-      <c r="H158" s="43"/>
-      <c r="I158" s="40"/>
-    </row>
-    <row r="159" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A159" s="47"/>
-      <c r="B159" s="12"/>
-      <c r="C159" s="18"/>
-      <c r="D159" s="41"/>
-      <c r="E159" s="40"/>
-      <c r="F159" s="47"/>
-      <c r="G159" s="42"/>
-      <c r="H159" s="43"/>
-      <c r="I159" s="40"/>
-    </row>
-    <row r="160" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A160" s="48"/>
-      <c r="B160" s="12"/>
-      <c r="C160" s="18"/>
-      <c r="D160" s="41"/>
-      <c r="E160" s="40"/>
-      <c r="F160" s="48"/>
-      <c r="G160" s="44"/>
-      <c r="H160" s="43"/>
-      <c r="I160" s="40"/>
+      <c r="C158" s="18"/>
+      <c r="D158" s="52"/>
+      <c r="E158" s="45"/>
+      <c r="F158" s="48"/>
+      <c r="G158" s="101"/>
+      <c r="H158" s="41"/>
+      <c r="I158" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="329">
+  <mergeCells count="323">
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="G2:H3"/>
+    <mergeCell ref="D145:E145"/>
+    <mergeCell ref="D146:E146"/>
+    <mergeCell ref="D148:E148"/>
+    <mergeCell ref="G155:I155"/>
+    <mergeCell ref="G156:I156"/>
+    <mergeCell ref="G157:I157"/>
+    <mergeCell ref="G158:I158"/>
+    <mergeCell ref="D149:E149"/>
+    <mergeCell ref="D150:E150"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="G151:I151"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="A153:I153"/>
+    <mergeCell ref="G154:I154"/>
+    <mergeCell ref="F142:F146"/>
+    <mergeCell ref="F148:F152"/>
+    <mergeCell ref="F154:F158"/>
+    <mergeCell ref="A147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="A141:I141"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="G144:I144"/>
+    <mergeCell ref="D151:E151"/>
+    <mergeCell ref="D152:E152"/>
+    <mergeCell ref="D154:E154"/>
+    <mergeCell ref="D155:E155"/>
+    <mergeCell ref="F138:F140"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="D156:E156"/>
+    <mergeCell ref="D157:E157"/>
+    <mergeCell ref="D158:E158"/>
+    <mergeCell ref="D140:E140"/>
+    <mergeCell ref="D142:E142"/>
+    <mergeCell ref="D143:E143"/>
+    <mergeCell ref="D144:E144"/>
+    <mergeCell ref="A138:A140"/>
+    <mergeCell ref="A142:A146"/>
+    <mergeCell ref="A148:A152"/>
+    <mergeCell ref="A154:A158"/>
+    <mergeCell ref="D138:E138"/>
+    <mergeCell ref="D139:E139"/>
+    <mergeCell ref="A120:A124"/>
+    <mergeCell ref="A126:A130"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="D120:E120"/>
+    <mergeCell ref="D123:E123"/>
+    <mergeCell ref="D126:E126"/>
+    <mergeCell ref="A83:I83"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="G87:I87"/>
+    <mergeCell ref="G88:I88"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="F126:F130"/>
+    <mergeCell ref="D127:E127"/>
+    <mergeCell ref="D128:E128"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="A90:A94"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="A102:A106"/>
+    <mergeCell ref="A108:A112"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="A66:A70"/>
+    <mergeCell ref="A72:A76"/>
+    <mergeCell ref="A78:A82"/>
+    <mergeCell ref="A107:I107"/>
+    <mergeCell ref="A84:A88"/>
+    <mergeCell ref="D105:E105"/>
+    <mergeCell ref="F84:F88"/>
+    <mergeCell ref="F91:F94"/>
+    <mergeCell ref="A89:I89"/>
+    <mergeCell ref="D90:I90"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="A71:I71"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D73:E73"/>
+    <mergeCell ref="F72:F76"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="D129:E129"/>
+    <mergeCell ref="D130:E130"/>
+    <mergeCell ref="D132:E135"/>
+    <mergeCell ref="F132:F135"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="G130:I130"/>
+    <mergeCell ref="A131:I131"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="A132:A136"/>
+    <mergeCell ref="D136:I136"/>
+    <mergeCell ref="A137:I137"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="A113:I113"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="D121:E121"/>
+    <mergeCell ref="D122:E122"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="G116:I116"/>
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="F120:F124"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="A125:I125"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="D116:E116"/>
+    <mergeCell ref="D117:E117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="F108:F112"/>
+    <mergeCell ref="D109:E112"/>
+    <mergeCell ref="D114:E114"/>
+    <mergeCell ref="F114:F118"/>
+    <mergeCell ref="D115:E115"/>
+    <mergeCell ref="D118:E118"/>
+    <mergeCell ref="A114:A118"/>
+    <mergeCell ref="P102:R102"/>
+    <mergeCell ref="A95:I95"/>
+    <mergeCell ref="D96:E96"/>
+    <mergeCell ref="F96:F100"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="M103:N103"/>
+    <mergeCell ref="P103:R103"/>
+    <mergeCell ref="D98:E98"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="O102:O106"/>
+    <mergeCell ref="D106:E106"/>
+    <mergeCell ref="M106:N106"/>
+    <mergeCell ref="M102:N102"/>
+    <mergeCell ref="D104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="P104:R104"/>
+    <mergeCell ref="P105:R105"/>
+    <mergeCell ref="P106:R106"/>
+    <mergeCell ref="D103:E103"/>
+    <mergeCell ref="M104:N104"/>
+    <mergeCell ref="M105:N105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="D97:E97"/>
+    <mergeCell ref="D100:E100"/>
+    <mergeCell ref="D102:E102"/>
+    <mergeCell ref="F102:F106"/>
+    <mergeCell ref="J102:J106"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="A101:I101"/>
+    <mergeCell ref="G102:I102"/>
+    <mergeCell ref="D93:E93"/>
+    <mergeCell ref="D94:E94"/>
+    <mergeCell ref="D84:E84"/>
+    <mergeCell ref="D85:E85"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="D91:E91"/>
+    <mergeCell ref="D92:E92"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="A42:A46"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:F46"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="F48:F52"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="F55:F57"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="A48:A52"/>
+    <mergeCell ref="A54:A58"/>
+    <mergeCell ref="F78:F82"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="G74:I74"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="G60:I60"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="A65:I65"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F60:F64"/>
+    <mergeCell ref="F66:F70"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="G62:I62"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:C2"/>
@@ -4417,311 +4646,6 @@
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A24:A28"/>
     <mergeCell ref="D24:E24"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="A65:I65"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="G67:I67"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F60:F64"/>
-    <mergeCell ref="F66:F70"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="F78:F82"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="G74:I74"/>
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="A77:I77"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="A53:I53"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="A59:I59"/>
-    <mergeCell ref="G60:I60"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="A42:A46"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:F46"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F48:F52"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F55:F57"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="A48:A52"/>
-    <mergeCell ref="A54:A58"/>
-    <mergeCell ref="D93:E93"/>
-    <mergeCell ref="D94:E94"/>
-    <mergeCell ref="D84:E84"/>
-    <mergeCell ref="D85:E85"/>
-    <mergeCell ref="D86:E86"/>
-    <mergeCell ref="D87:E87"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="D91:E91"/>
-    <mergeCell ref="D92:E92"/>
-    <mergeCell ref="M104:N104"/>
-    <mergeCell ref="M105:N105"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="D97:E97"/>
-    <mergeCell ref="D100:E100"/>
-    <mergeCell ref="D102:E102"/>
-    <mergeCell ref="F102:F106"/>
-    <mergeCell ref="J102:J106"/>
-    <mergeCell ref="G100:I100"/>
-    <mergeCell ref="A101:I101"/>
-    <mergeCell ref="G102:I102"/>
-    <mergeCell ref="A114:A118"/>
-    <mergeCell ref="P102:R102"/>
-    <mergeCell ref="A95:I95"/>
-    <mergeCell ref="D96:E96"/>
-    <mergeCell ref="F96:F100"/>
-    <mergeCell ref="G96:I96"/>
-    <mergeCell ref="G97:I97"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="M103:N103"/>
-    <mergeCell ref="P103:R103"/>
-    <mergeCell ref="D98:E98"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="O102:O106"/>
-    <mergeCell ref="D106:E106"/>
-    <mergeCell ref="M106:N106"/>
-    <mergeCell ref="M102:N102"/>
-    <mergeCell ref="D104:E104"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="P104:R104"/>
-    <mergeCell ref="P105:R105"/>
-    <mergeCell ref="P106:R106"/>
-    <mergeCell ref="D103:E103"/>
-    <mergeCell ref="D116:E116"/>
-    <mergeCell ref="D117:E117"/>
-    <mergeCell ref="G117:I117"/>
-    <mergeCell ref="G118:I118"/>
-    <mergeCell ref="F108:F112"/>
-    <mergeCell ref="D109:E112"/>
-    <mergeCell ref="D114:E114"/>
-    <mergeCell ref="F114:F118"/>
-    <mergeCell ref="D115:E115"/>
-    <mergeCell ref="D118:E118"/>
-    <mergeCell ref="A137:I137"/>
-    <mergeCell ref="G138:I139"/>
-    <mergeCell ref="G108:I108"/>
-    <mergeCell ref="G109:I109"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="G111:I111"/>
-    <mergeCell ref="G112:I112"/>
-    <mergeCell ref="A113:I113"/>
-    <mergeCell ref="G114:I114"/>
-    <mergeCell ref="D121:E121"/>
-    <mergeCell ref="D122:E122"/>
-    <mergeCell ref="G123:I123"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="G124:I124"/>
-    <mergeCell ref="G115:I115"/>
-    <mergeCell ref="G116:I116"/>
-    <mergeCell ref="A119:I119"/>
-    <mergeCell ref="F120:F124"/>
-    <mergeCell ref="G120:I120"/>
-    <mergeCell ref="G121:I121"/>
-    <mergeCell ref="G122:I122"/>
-    <mergeCell ref="A125:I125"/>
-    <mergeCell ref="G126:I126"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="D129:E129"/>
-    <mergeCell ref="D130:E130"/>
-    <mergeCell ref="D132:E135"/>
-    <mergeCell ref="F132:F135"/>
-    <mergeCell ref="G134:I134"/>
-    <mergeCell ref="G135:I135"/>
-    <mergeCell ref="G127:I127"/>
-    <mergeCell ref="G128:I128"/>
-    <mergeCell ref="G129:I129"/>
-    <mergeCell ref="G130:I130"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="G132:I132"/>
-    <mergeCell ref="G133:I133"/>
-    <mergeCell ref="A132:A136"/>
-    <mergeCell ref="D136:I136"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A12:A16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="G69:I69"/>
-    <mergeCell ref="G70:I70"/>
-    <mergeCell ref="A71:I71"/>
-    <mergeCell ref="G72:I72"/>
-    <mergeCell ref="G73:I73"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="F72:F76"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="A90:A94"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="A102:A106"/>
-    <mergeCell ref="A108:A112"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="A66:A70"/>
-    <mergeCell ref="A72:A76"/>
-    <mergeCell ref="A78:A82"/>
-    <mergeCell ref="A107:I107"/>
-    <mergeCell ref="A84:A88"/>
-    <mergeCell ref="D105:E105"/>
-    <mergeCell ref="F84:F88"/>
-    <mergeCell ref="F91:F94"/>
-    <mergeCell ref="A89:I89"/>
-    <mergeCell ref="D90:I90"/>
-    <mergeCell ref="G91:I91"/>
-    <mergeCell ref="G92:I92"/>
-    <mergeCell ref="G93:I93"/>
-    <mergeCell ref="G94:I94"/>
-    <mergeCell ref="A120:A124"/>
-    <mergeCell ref="A126:A130"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="D78:E78"/>
-    <mergeCell ref="D79:E79"/>
-    <mergeCell ref="D80:E80"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="D82:E82"/>
-    <mergeCell ref="D120:E120"/>
-    <mergeCell ref="D123:E123"/>
-    <mergeCell ref="D126:E126"/>
-    <mergeCell ref="A83:I83"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="G85:I85"/>
-    <mergeCell ref="G86:I86"/>
-    <mergeCell ref="G87:I87"/>
-    <mergeCell ref="G88:I88"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="F126:F130"/>
-    <mergeCell ref="D127:E127"/>
-    <mergeCell ref="D128:E128"/>
-    <mergeCell ref="D158:E158"/>
-    <mergeCell ref="D159:E159"/>
-    <mergeCell ref="D160:E160"/>
-    <mergeCell ref="D142:E142"/>
-    <mergeCell ref="D144:E144"/>
-    <mergeCell ref="D145:E145"/>
-    <mergeCell ref="D146:E146"/>
-    <mergeCell ref="A138:A142"/>
-    <mergeCell ref="A144:A148"/>
-    <mergeCell ref="A150:A154"/>
-    <mergeCell ref="A156:A160"/>
-    <mergeCell ref="D138:E139"/>
-    <mergeCell ref="D140:E140"/>
-    <mergeCell ref="D141:E141"/>
-    <mergeCell ref="G142:I142"/>
-    <mergeCell ref="A143:I143"/>
-    <mergeCell ref="G144:I144"/>
-    <mergeCell ref="G145:I145"/>
-    <mergeCell ref="G146:I146"/>
-    <mergeCell ref="D153:E153"/>
-    <mergeCell ref="D154:E154"/>
-    <mergeCell ref="D156:E156"/>
-    <mergeCell ref="D157:E157"/>
-    <mergeCell ref="F138:F142"/>
-    <mergeCell ref="G147:I147"/>
-    <mergeCell ref="G148:I148"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="G2:H3"/>
-    <mergeCell ref="D147:E147"/>
-    <mergeCell ref="D148:E148"/>
-    <mergeCell ref="D150:E150"/>
-    <mergeCell ref="G157:I157"/>
-    <mergeCell ref="G158:I158"/>
-    <mergeCell ref="G159:I159"/>
-    <mergeCell ref="G160:I160"/>
-    <mergeCell ref="D151:E151"/>
-    <mergeCell ref="D152:E152"/>
-    <mergeCell ref="G152:I152"/>
-    <mergeCell ref="G153:I153"/>
-    <mergeCell ref="G154:I154"/>
-    <mergeCell ref="A155:I155"/>
-    <mergeCell ref="G156:I156"/>
-    <mergeCell ref="F144:F148"/>
-    <mergeCell ref="F150:F154"/>
-    <mergeCell ref="F156:F160"/>
-    <mergeCell ref="A149:I149"/>
-    <mergeCell ref="G150:I150"/>
-    <mergeCell ref="G151:I151"/>
-    <mergeCell ref="G140:I140"/>
-    <mergeCell ref="G141:I141"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>